<commit_message>
Toevoeging normbandbreedtes voor lelysphere
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/luchtzuiveringssysteem/luchtzuiveringssysteem.xlsx
+++ b/src/main/resources/be/vlaanderen/omgeving/data/id/conceptscheme/luchtzuiveringssysteem/luchtzuiveringssysteem.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC92"/>
+  <dimension ref="A1:AC97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2626,7 +2626,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_17</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2644,7 +2644,7 @@
         <v>null</v>
       </c>
       <c r="G26" t="str">
-        <v>Zuurtegraad waswater &gt; 8,5 (S1 systeem)</v>
+        <v>Geleidbaarheid waswater &gt; 280mS/cm (lelysphere)</v>
       </c>
       <c r="H26" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
@@ -2653,19 +2653,19 @@
         <v>Boven maximum grenswaarde</v>
       </c>
       <c r="J26" t="str">
-        <v>De zuurtegraad van het waswater is groter dan 8,5</v>
+        <v>De geleidbaarheid is groter dan 280mS/cm</v>
       </c>
       <c r="K26" t="str">
-        <v>De zuurtegraad van het waswater is groter dan 8,5|&gt; 8,5</v>
+        <v>De geleidbaarheid is groter dan 280mS/cm|&gt; 280</v>
       </c>
       <c r="L26" t="str">
-        <v>&gt; 8,5</v>
+        <v>&gt; 280</v>
       </c>
       <c r="M26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N26" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="O26" t="str">
         <v>null</v>
@@ -2674,7 +2674,7 @@
         <v>null</v>
       </c>
       <c r="Q26" t="str">
-        <v>8.5</v>
+        <v>280</v>
       </c>
       <c r="R26" t="str">
         <v>null</v>
@@ -2715,7 +2715,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_18</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2733,7 +2733,7 @@
         <v>null</v>
       </c>
       <c r="G27" t="str">
-        <v>Geleidbaarheid waswater &gt; maximale waarde (S1 systeem)</v>
+        <v>Geleidbaarheid waswater afwijking naar boven &gt; 40mS/cm (lelysphere)</v>
       </c>
       <c r="H27" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
@@ -2745,13 +2745,13 @@
         <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K27" t="str">
-        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.|&gt; waarde technische fiche</v>
+        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.|&gt; 40mS/cm + waarde technische fiche (afwijking &gt; 40mS/cm)</v>
       </c>
       <c r="L27" t="str">
-        <v>&gt; waarde technische fiche</v>
+        <v>&gt; 40mS/cm + waarde technische fiche (afwijking &gt; 40mS/cm)</v>
       </c>
       <c r="M27" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N27" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
@@ -2763,7 +2763,7 @@
         <v>som</v>
       </c>
       <c r="Q27" t="str">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="R27" t="str">
         <v>null</v>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_4</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_19</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2822,7 +2822,7 @@
         <v>null</v>
       </c>
       <c r="G28" t="str">
-        <v>Waswaterdebiet afwijking naar beneden &gt; 20% (S1 systeem)</v>
+        <v>Waswaterdebiet afwijking naar beneden &gt; 20% (lelysphere)</v>
       </c>
       <c r="H28" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
@@ -2840,13 +2840,13 @@
         <v>&lt; 0,8 x waarde technische fiche (afwijking &gt; 20%)</v>
       </c>
       <c r="M28" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N28" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
       </c>
       <c r="O28" t="str">
-        <v>0.8</v>
+        <v>0,8</v>
       </c>
       <c r="P28" t="str">
         <v>product</v>
@@ -2893,7 +2893,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_5</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_2</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -2911,37 +2911,37 @@
         <v>null</v>
       </c>
       <c r="G29" t="str">
-        <v>Spuiwaterdebiet afwijking naar beneden &gt; 10% (S1 systeem)</v>
+        <v>Zuurtegraad waswater &gt; 8,5 (S1 systeem)</v>
       </c>
       <c r="H29" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I29" t="str">
-        <v>Onder minimum grenswaarde</v>
+        <v>Boven maximum grenswaarde</v>
       </c>
       <c r="J29" t="str">
-        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
+        <v>De zuurtegraad van het waswater is groter dan 8,5</v>
       </c>
       <c r="K29" t="str">
-        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
+        <v>De zuurtegraad van het waswater is groter dan 8,5|&gt; 8,5</v>
       </c>
       <c r="L29" t="str">
-        <v>&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
+        <v>&gt; 8,5</v>
       </c>
       <c r="M29" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N29" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
       </c>
       <c r="O29" t="str">
-        <v>0.9</v>
+        <v>null</v>
       </c>
       <c r="P29" t="str">
-        <v>product</v>
+        <v>null</v>
       </c>
       <c r="Q29" t="str">
-        <v>null</v>
+        <v>8.5</v>
       </c>
       <c r="R29" t="str">
         <v>null</v>
@@ -2982,7 +2982,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_6</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_20</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3000,7 +3000,7 @@
         <v>null</v>
       </c>
       <c r="G30" t="str">
-        <v>Drukval afwijking naar beneden &gt; 40% (S1 systeem)</v>
+        <v>Spuiwaterdebiet afwijking naar beneden &gt; 10% (lelysphere)</v>
       </c>
       <c r="H30" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
@@ -3009,22 +3009,22 @@
         <v>Onder minimum grenswaarde</v>
       </c>
       <c r="J30" t="str">
-        <v>De drukval wijkt meer dan 40% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
+        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K30" t="str">
-        <v>De drukval wijkt meer dan 40% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,6 x waarde technische fiche (afwijking &gt; 40%)</v>
+        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
       </c>
       <c r="L30" t="str">
-        <v>&lt; 0,6 x waarde technische fiche (afwijking &gt; 40%)</v>
+        <v>&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
       </c>
       <c r="M30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N30" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
       </c>
       <c r="O30" t="str">
-        <v>0.6</v>
+        <v>0,9</v>
       </c>
       <c r="P30" t="str">
         <v>product</v>
@@ -3071,7 +3071,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_7</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_21</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3089,37 +3089,37 @@
         <v>null</v>
       </c>
       <c r="G31" t="str">
-        <v>Drukval afwijking naar boven &gt; 40% (S1 systeem)</v>
+        <v>Elektriciteitsverbruik van de waswaterpomp &lt; 1 kWh (lelysphere)</v>
       </c>
       <c r="H31" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I31" t="str">
-        <v>Boven maximum grenswaarde</v>
+        <v>Onder minimum grenswaarde</v>
       </c>
       <c r="J31" t="str">
-        <v>De drukval wijkt meer dan 40% naar boven af van de operationele waarde die op de technische fiche vermeld staat.</v>
+        <v>Het elektriciteitsverbruik van de waswaterpomp is kleiner dan  1 kWh</v>
       </c>
       <c r="K31" t="str">
-        <v>De drukval wijkt meer dan 40% naar boven af van de operationele waarde die op de technische fiche vermeld staat.|&gt; 1,4 x waarde technische fiche (afwijking &gt; 40%)</v>
+        <v>Het elektriciteitsverbruik van de waswaterpomp is kleiner dan  1 kWh|&lt; 1</v>
       </c>
       <c r="L31" t="str">
-        <v>&gt; 1,4 x waarde technische fiche (afwijking &gt; 40%)</v>
+        <v>&lt; 1</v>
       </c>
       <c r="M31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N31" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
       </c>
       <c r="O31" t="str">
-        <v>null</v>
+        <v>1</v>
       </c>
       <c r="P31" t="str">
-        <v>product</v>
+        <v>null</v>
       </c>
       <c r="Q31" t="str">
-        <v>1.4</v>
+        <v>null</v>
       </c>
       <c r="R31" t="str">
         <v>null</v>
@@ -3160,7 +3160,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_8</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_3</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3178,7 +3178,7 @@
         <v>null</v>
       </c>
       <c r="G32" t="str">
-        <v>Zuurtegraad waswater afwijking naar boven &gt; 1 pH-eenheid (S2 systeem)</v>
+        <v>Geleidbaarheid waswater &gt; maximale waarde (S1 systeem)</v>
       </c>
       <c r="H32" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
@@ -3187,19 +3187,19 @@
         <v>Boven maximum grenswaarde</v>
       </c>
       <c r="J32" t="str">
-        <v>De zuurtegraad van het waswater wijkt meer dan 1 pH-eenheid naar boven af van de operationele waarde die op de technische fiche vermeld staat.</v>
+        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K32" t="str">
-        <v>De zuurtegraad van het waswater wijkt meer dan 1 pH-eenheid naar boven af van de operationele waarde die op de technische fiche vermeld staat.|&gt; 1 pH + waarde technische fiche (afwijking &gt; 1pH)</v>
+        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.|&gt; waarde technische fiche</v>
       </c>
       <c r="L32" t="str">
-        <v>&gt; 1 pH + waarde technische fiche (afwijking &gt; 1pH)</v>
+        <v>&gt; waarde technische fiche</v>
       </c>
       <c r="M32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N32" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="O32" t="str">
         <v>null</v>
@@ -3208,7 +3208,7 @@
         <v>som</v>
       </c>
       <c r="Q32" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R32" t="str">
         <v>null</v>
@@ -3249,7 +3249,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_9</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_4</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -3267,37 +3267,37 @@
         <v>null</v>
       </c>
       <c r="G33" t="str">
-        <v>Geleidbaarheid waswater &gt; maximale waarde (S2 systeem)</v>
+        <v>Waswaterdebiet afwijking naar beneden &gt; 20% (S1 systeem)</v>
       </c>
       <c r="H33" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I33" t="str">
-        <v>Boven maximum grenswaarde</v>
+        <v>Onder minimum grenswaarde</v>
       </c>
       <c r="J33" t="str">
-        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.</v>
+        <v>Het waswaterdebiet wijkt meer dan 20% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K33" t="str">
-        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.|&gt; waarde technische fiche</v>
+        <v>Het waswaterdebiet wijkt meer dan 20% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,8 x waarde technische fiche (afwijking &gt; 20%)</v>
       </c>
       <c r="L33" t="str">
-        <v>&gt; waarde technische fiche</v>
+        <v>&lt; 0,8 x waarde technische fiche (afwijking &gt; 20%)</v>
       </c>
       <c r="M33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N33" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
       </c>
       <c r="O33" t="str">
-        <v>null</v>
+        <v>0.8</v>
       </c>
       <c r="P33" t="str">
-        <v>som</v>
+        <v>product</v>
       </c>
       <c r="Q33" t="str">
-        <v>0</v>
+        <v>null</v>
       </c>
       <c r="R33" t="str">
         <v>null</v>
@@ -3338,10 +3338,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_5</v>
       </c>
       <c r="B34" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
         <v>null</v>
@@ -3350,52 +3350,52 @@
         <v>null</v>
       </c>
       <c r="E34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="F34" t="str">
         <v>null</v>
       </c>
       <c r="G34" t="str">
-        <v>Biobedspoelwaterproductie</v>
+        <v>Spuiwaterdebiet afwijking naar beneden &gt; 10% (S1 systeem)</v>
       </c>
       <c r="H34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I34" t="str">
-        <v>null</v>
+        <v>Onder minimum grenswaarde</v>
       </c>
       <c r="J34" t="str">
-        <v>null</v>
+        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K34" t="str">
-        <v>null</v>
+        <v>Het spuiwaterdebiet wijkt meer dan 10% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
       </c>
       <c r="L34" t="str">
-        <v>null</v>
+        <v>&lt; 0,9 x waarde technische fiche (afwijking &gt; 10%)</v>
       </c>
       <c r="M34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N34" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
       </c>
       <c r="O34" t="str">
-        <v>null</v>
+        <v>0.9</v>
       </c>
       <c r="P34" t="str">
-        <v>null</v>
+        <v>product</v>
       </c>
       <c r="Q34" t="str">
         <v>null</v>
       </c>
       <c r="R34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>null</v>
       </c>
       <c r="S34" t="str">
-        <v>http://qudt.org/vocab/quantitykind/Volume</v>
+        <v>null</v>
       </c>
       <c r="T34" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
+        <v>null</v>
       </c>
       <c r="U34" t="str">
         <v>null</v>
@@ -3427,10 +3427,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_6</v>
       </c>
       <c r="B35" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
         <v>null</v>
@@ -3439,52 +3439,52 @@
         <v>null</v>
       </c>
       <c r="E35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="F35" t="str">
         <v>null</v>
       </c>
       <c r="G35" t="str">
-        <v>Biobedspuiwaterproductie</v>
+        <v>Drukval afwijking naar beneden &gt; 40% (S1 systeem)</v>
       </c>
       <c r="H35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I35" t="str">
-        <v>null</v>
+        <v>Onder minimum grenswaarde</v>
       </c>
       <c r="J35" t="str">
-        <v>null</v>
+        <v>De drukval wijkt meer dan 40% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K35" t="str">
-        <v>null</v>
+        <v>De drukval wijkt meer dan 40% naar beneden af van de operationele waarde die op de technische fiche vermeld staat.|&lt; 0,6 x waarde technische fiche (afwijking &gt; 40%)</v>
       </c>
       <c r="L35" t="str">
-        <v>null</v>
+        <v>&lt; 0,6 x waarde technische fiche (afwijking &gt; 40%)</v>
       </c>
       <c r="M35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N35" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
       </c>
       <c r="O35" t="str">
-        <v>null</v>
+        <v>0.6</v>
       </c>
       <c r="P35" t="str">
-        <v>null</v>
+        <v>product</v>
       </c>
       <c r="Q35" t="str">
         <v>null</v>
       </c>
       <c r="R35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater</v>
+        <v>null</v>
       </c>
       <c r="S35" t="str">
-        <v>http://qudt.org/vocab/quantitykind/Volume</v>
+        <v>null</v>
       </c>
       <c r="T35" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0050</v>
+        <v>null</v>
       </c>
       <c r="U35" t="str">
         <v>null</v>
@@ -3516,64 +3516,64 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_7</v>
+      </c>
+      <c r="B36" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+      </c>
+      <c r="C36" t="str">
+        <v>null</v>
+      </c>
+      <c r="D36" t="str">
+        <v>null</v>
+      </c>
+      <c r="E36" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
+      </c>
+      <c r="F36" t="str">
+        <v>null</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Drukval afwijking naar boven &gt; 40% (S1 systeem)</v>
+      </c>
+      <c r="H36" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Boven maximum grenswaarde</v>
+      </c>
+      <c r="J36" t="str">
+        <v>De drukval wijkt meer dan 40% naar boven af van de operationele waarde die op de technische fiche vermeld staat.</v>
+      </c>
+      <c r="K36" t="str">
+        <v>De drukval wijkt meer dan 40% naar boven af van de operationele waarde die op de technische fiche vermeld staat.|&gt; 1,4 x waarde technische fiche (afwijking &gt; 40%)</v>
+      </c>
+      <c r="L36" t="str">
+        <v>&gt; 1,4 x waarde technische fiche (afwijking &gt; 40%)</v>
+      </c>
+      <c r="M36" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+      </c>
+      <c r="N36" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
       </c>
-      <c r="B36" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
-      </c>
-      <c r="C36" t="str">
-        <v>null</v>
-      </c>
-      <c r="D36" t="str">
-        <v>null</v>
-      </c>
-      <c r="E36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
-      </c>
-      <c r="F36" t="str">
-        <v>null</v>
-      </c>
-      <c r="G36" t="str">
-        <v>Drukval over het systeem</v>
-      </c>
-      <c r="H36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
-      </c>
-      <c r="I36" t="str">
-        <v>null</v>
-      </c>
-      <c r="J36" t="str">
-        <v>null</v>
-      </c>
-      <c r="K36" t="str">
-        <v>null</v>
-      </c>
-      <c r="L36" t="str">
-        <v>null</v>
-      </c>
-      <c r="M36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
-      </c>
-      <c r="N36" t="str">
-        <v>null</v>
-      </c>
       <c r="O36" t="str">
         <v>null</v>
       </c>
       <c r="P36" t="str">
-        <v>null</v>
+        <v>product</v>
       </c>
       <c r="Q36" t="str">
-        <v>null</v>
+        <v>1.4</v>
       </c>
       <c r="R36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/lucht</v>
+        <v>null</v>
       </c>
       <c r="S36" t="str">
-        <v>http://qudt.org/vocab/quantitykind/VaporPressure</v>
+        <v>null</v>
       </c>
       <c r="T36" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0329</v>
+        <v>null</v>
       </c>
       <c r="U36" t="str">
         <v>null</v>
@@ -3605,10 +3605,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_8</v>
       </c>
       <c r="B37" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C37" t="str">
         <v>null</v>
@@ -3617,49 +3617,49 @@
         <v>null</v>
       </c>
       <c r="E37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="F37" t="str">
         <v>null</v>
       </c>
       <c r="G37" t="str">
-        <v>Elektriciteitsverbruik van de waswaterpomp(en)</v>
+        <v>Zuurtegraad waswater afwijking naar boven &gt; 1 pH-eenheid (S2 systeem)</v>
       </c>
       <c r="H37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="I37" t="str">
-        <v>null</v>
+        <v>Boven maximum grenswaarde</v>
       </c>
       <c r="J37" t="str">
-        <v>null</v>
+        <v>De zuurtegraad van het waswater wijkt meer dan 1 pH-eenheid naar boven af van de operationele waarde die op de technische fiche vermeld staat.</v>
       </c>
       <c r="K37" t="str">
-        <v>null</v>
+        <v>De zuurtegraad van het waswater wijkt meer dan 1 pH-eenheid naar boven af van de operationele waarde die op de technische fiche vermeld staat.|&gt; 1 pH + waarde technische fiche (afwijking &gt; 1pH)</v>
       </c>
       <c r="L37" t="str">
-        <v>null</v>
+        <v>&gt; 1 pH + waarde technische fiche (afwijking &gt; 1pH)</v>
       </c>
       <c r="M37" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N37" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
       </c>
       <c r="O37" t="str">
         <v>null</v>
       </c>
       <c r="P37" t="str">
-        <v>null</v>
+        <v>som</v>
       </c>
       <c r="Q37" t="str">
-        <v>null</v>
+        <v>1</v>
       </c>
       <c r="R37" t="str">
         <v>null</v>
       </c>
       <c r="S37" t="str">
-        <v>http://qudt.org/vocab/quantitykind/Energy</v>
+        <v>null</v>
       </c>
       <c r="T37" t="str">
         <v>null</v>
@@ -3694,64 +3694,64 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_9</v>
+      </c>
+      <c r="B38" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+      </c>
+      <c r="C38" t="str">
+        <v>null</v>
+      </c>
+      <c r="D38" t="str">
+        <v>null</v>
+      </c>
+      <c r="E38" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
+      </c>
+      <c r="F38" t="str">
+        <v>null</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Geleidbaarheid waswater &gt; maximale waarde (S2 systeem)</v>
+      </c>
+      <c r="H38" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Boven maximum grenswaarde</v>
+      </c>
+      <c r="J38" t="str">
+        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.</v>
+      </c>
+      <c r="K38" t="str">
+        <v>De geleidbaarheid is groter dan de maximale operationele waarde die op de technische fiche vermeld staat.|&gt; waarde technische fiche</v>
+      </c>
+      <c r="L38" t="str">
+        <v>&gt; waarde technische fiche</v>
+      </c>
+      <c r="M38" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+      </c>
+      <c r="N38" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
-      <c r="B38" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
-      </c>
-      <c r="C38" t="str">
-        <v>null</v>
-      </c>
-      <c r="D38" t="str">
-        <v>null</v>
-      </c>
-      <c r="E38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
-      </c>
-      <c r="F38" t="str">
-        <v>null</v>
-      </c>
-      <c r="G38" t="str">
-        <v>Geleidbaarheid van het waswater</v>
-      </c>
-      <c r="H38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
-      </c>
-      <c r="I38" t="str">
-        <v>null</v>
-      </c>
-      <c r="J38" t="str">
-        <v>null</v>
-      </c>
-      <c r="K38" t="str">
-        <v>null</v>
-      </c>
-      <c r="L38" t="str">
-        <v>null</v>
-      </c>
-      <c r="M38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
-      </c>
-      <c r="N38" t="str">
-        <v>null</v>
-      </c>
       <c r="O38" t="str">
         <v>null</v>
       </c>
       <c r="P38" t="str">
-        <v>null</v>
+        <v>som</v>
       </c>
       <c r="Q38" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>null</v>
       </c>
       <c r="S38" t="str">
-        <v>http://qudt.org/vocab/quantitykind/Conductivity</v>
+        <v>null</v>
       </c>
       <c r="T38" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0010</v>
+        <v>null</v>
       </c>
       <c r="U38" t="str">
         <v>null</v>
@@ -3783,7 +3783,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie</v>
       </c>
       <c r="B39" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -3801,7 +3801,7 @@
         <v>null</v>
       </c>
       <c r="G39" t="str">
-        <v>Spuiwaterproductie</v>
+        <v>Biobedspoelwaterproductie</v>
       </c>
       <c r="H39" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -3819,7 +3819,7 @@
         <v>null</v>
       </c>
       <c r="M39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N39" t="str">
         <v>null</v>
@@ -3834,13 +3834,13 @@
         <v>null</v>
       </c>
       <c r="R39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S39" t="str">
         <v>http://qudt.org/vocab/quantitykind/Volume</v>
       </c>
       <c r="T39" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0050</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
       </c>
       <c r="U39" t="str">
         <v>null</v>
@@ -3872,7 +3872,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie</v>
       </c>
       <c r="B40" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -3890,7 +3890,7 @@
         <v>null</v>
       </c>
       <c r="G40" t="str">
-        <v>Stalbezetting</v>
+        <v>Biobedspuiwaterproductie</v>
       </c>
       <c r="H40" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -3908,7 +3908,7 @@
         <v>null</v>
       </c>
       <c r="M40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N40" t="str">
         <v>null</v>
@@ -3923,16 +3923,16 @@
         <v>null</v>
       </c>
       <c r="R40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/stal</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater</v>
       </c>
       <c r="S40" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/Volume</v>
       </c>
       <c r="T40" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0050</v>
       </c>
       <c r="U40" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>null</v>
       </c>
       <c r="V40" t="str">
         <v>null</v>
@@ -3961,7 +3961,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
       </c>
       <c r="B41" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -3979,7 +3979,7 @@
         <v>null</v>
       </c>
       <c r="G41" t="str">
-        <v>SysteemStatus</v>
+        <v>Drukval over het systeem</v>
       </c>
       <c r="H41" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -4012,16 +4012,16 @@
         <v>null</v>
       </c>
       <c r="R41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/hetelektronischmonitoringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/lucht</v>
       </c>
       <c r="S41" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/VaporPressure</v>
       </c>
       <c r="T41" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0329</v>
       </c>
       <c r="U41" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>null</v>
       </c>
       <c r="V41" t="str">
         <v>null</v>
@@ -4050,7 +4050,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
       </c>
       <c r="B42" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -4068,7 +4068,7 @@
         <v>null</v>
       </c>
       <c r="G42" t="str">
-        <v>Waswaterdebiet over het waspakket</v>
+        <v>Elektriciteitsverbruik van de waswaterpomp(en)</v>
       </c>
       <c r="H42" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -4086,7 +4086,7 @@
         <v>null</v>
       </c>
       <c r="M42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N42" t="str">
         <v>null</v>
@@ -4101,13 +4101,13 @@
         <v>null</v>
       </c>
       <c r="R42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>null</v>
       </c>
       <c r="S42" t="str">
-        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
+        <v>http://qudt.org/vocab/quantitykind/Energy</v>
       </c>
       <c r="T42" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
+        <v>null</v>
       </c>
       <c r="U42" t="str">
         <v>null</v>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="B43" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -4157,7 +4157,7 @@
         <v>null</v>
       </c>
       <c r="G43" t="str">
-        <v>Waswaterdebiet van de bevloeiing van het vulmateriaal</v>
+        <v>Geleidbaarheid van het waswater</v>
       </c>
       <c r="H43" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -4175,7 +4175,7 @@
         <v>null</v>
       </c>
       <c r="M43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N43" t="str">
         <v>null</v>
@@ -4193,10 +4193,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S43" t="str">
-        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
+        <v>http://qudt.org/vocab/quantitykind/Conductivity</v>
       </c>
       <c r="T43" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0010</v>
       </c>
       <c r="U43" t="str">
         <v>null</v>
@@ -4228,7 +4228,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
       </c>
       <c r="B44" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -4246,7 +4246,7 @@
         <v>null</v>
       </c>
       <c r="G44" t="str">
-        <v>Waswaterdebiet van de voorbevochtiging van de ingaande stallucht</v>
+        <v>Spuiwaterproductie</v>
       </c>
       <c r="H44" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -4264,7 +4264,7 @@
         <v>null</v>
       </c>
       <c r="M44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N44" t="str">
         <v>null</v>
@@ -4279,13 +4279,13 @@
         <v>null</v>
       </c>
       <c r="R44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater</v>
       </c>
       <c r="S44" t="str">
-        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
+        <v>http://qudt.org/vocab/quantitykind/Volume</v>
       </c>
       <c r="T44" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0050</v>
       </c>
       <c r="U44" t="str">
         <v>null</v>
@@ -4317,7 +4317,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting</v>
       </c>
       <c r="B45" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
@@ -4335,7 +4335,7 @@
         <v>null</v>
       </c>
       <c r="G45" t="str">
-        <v>Zuurtegraad van het waswater</v>
+        <v>Stalbezetting</v>
       </c>
       <c r="H45" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
@@ -4353,7 +4353,7 @@
         <v>null</v>
       </c>
       <c r="M45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N45" t="str">
         <v>null</v>
@@ -4368,16 +4368,16 @@
         <v>null</v>
       </c>
       <c r="R45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/stal</v>
       </c>
       <c r="S45" t="str">
-        <v>http://qudt.org/vocab/quantitykind/Acidity</v>
+        <v>null</v>
       </c>
       <c r="T45" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0076</v>
+        <v>null</v>
       </c>
       <c r="U45" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
       </c>
       <c r="V45" t="str">
         <v>null</v>
@@ -4406,10 +4406,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
       <c r="B46" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
       </c>
       <c r="C46" t="str">
         <v>null</v>
@@ -4418,16 +4418,16 @@
         <v>null</v>
       </c>
       <c r="E46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="F46" t="str">
         <v>null</v>
       </c>
       <c r="G46" t="str">
-        <v>Zuurtegraad waswater S1 systeem</v>
+        <v>SysteemStatus</v>
       </c>
       <c r="H46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="I46" t="str">
         <v>null</v>
@@ -4442,22 +4442,22 @@
         <v>null</v>
       </c>
       <c r="M46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N46" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
+        <v>null</v>
       </c>
       <c r="O46" t="str">
-        <v>8.5</v>
+        <v>null</v>
       </c>
       <c r="P46" t="str">
         <v>null</v>
       </c>
       <c r="Q46" t="str">
-        <v>6</v>
+        <v>null</v>
       </c>
       <c r="R46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/hetelektronischmonitoringssysteem</v>
       </c>
       <c r="S46" t="str">
         <v>null</v>
@@ -4466,13 +4466,13 @@
         <v>null</v>
       </c>
       <c r="U46" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="V46" t="str">
-        <v>maximum</v>
+        <v>null</v>
       </c>
       <c r="W46" t="str">
-        <v>true</v>
+        <v>null</v>
       </c>
       <c r="X46" t="str">
         <v>null</v>
@@ -4495,10 +4495,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_10</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
       </c>
       <c r="B47" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
       </c>
       <c r="C47" t="str">
         <v>null</v>
@@ -4507,16 +4507,16 @@
         <v>null</v>
       </c>
       <c r="E47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="F47" t="str">
         <v>null</v>
       </c>
       <c r="G47" t="str">
-        <v>Drukval S2 systeem</v>
+        <v>Waswaterdebiet over het waspakket</v>
       </c>
       <c r="H47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="I47" t="str">
         <v>null</v>
@@ -4531,37 +4531,37 @@
         <v>null</v>
       </c>
       <c r="M47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N47" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
+        <v>null</v>
       </c>
       <c r="O47" t="str">
-        <v>500</v>
+        <v>null</v>
       </c>
       <c r="P47" t="str">
         <v>null</v>
       </c>
       <c r="Q47" t="str">
-        <v>0</v>
+        <v>null</v>
       </c>
       <c r="R47" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S47" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
       </c>
       <c r="T47" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
       </c>
       <c r="U47" t="str">
         <v>null</v>
       </c>
       <c r="V47" t="str">
-        <v>exact</v>
+        <v>null</v>
       </c>
       <c r="W47" t="str">
-        <v>true</v>
+        <v>null</v>
       </c>
       <c r="X47" t="str">
         <v>null</v>
@@ -4584,10 +4584,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_11</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing</v>
       </c>
       <c r="B48" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
       </c>
       <c r="C48" t="str">
         <v>null</v>
@@ -4596,16 +4596,16 @@
         <v>null</v>
       </c>
       <c r="E48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="F48" t="str">
         <v>null</v>
       </c>
       <c r="G48" t="str">
-        <v>Waswaterdebiet voorbevochtiging S3 systeem</v>
+        <v>Waswaterdebiet van de bevloeiing van het vulmateriaal</v>
       </c>
       <c r="H48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="I48" t="str">
         <v>null</v>
@@ -4623,7 +4623,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N48" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging</v>
+        <v>null</v>
       </c>
       <c r="O48" t="str">
         <v>null</v>
@@ -4632,25 +4632,25 @@
         <v>null</v>
       </c>
       <c r="Q48" t="str">
-        <v>0</v>
+        <v>null</v>
       </c>
       <c r="R48" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S48" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
       </c>
       <c r="T48" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
       </c>
       <c r="U48" t="str">
         <v>null</v>
       </c>
       <c r="V48" t="str">
-        <v>minimum</v>
+        <v>null</v>
       </c>
       <c r="W48" t="str">
-        <v>true</v>
+        <v>null</v>
       </c>
       <c r="X48" t="str">
         <v>null</v>
@@ -4673,10 +4673,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_12</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging</v>
       </c>
       <c r="B49" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
       </c>
       <c r="C49" t="str">
         <v>null</v>
@@ -4685,16 +4685,16 @@
         <v>null</v>
       </c>
       <c r="E49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="F49" t="str">
         <v>null</v>
       </c>
       <c r="G49" t="str">
-        <v>Waswaterdebiet bevloeiing S3 systeem</v>
+        <v>Waswaterdebiet van de voorbevochtiging van de ingaande stallucht</v>
       </c>
       <c r="H49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="I49" t="str">
         <v>null</v>
@@ -4712,7 +4712,7 @@
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N49" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing</v>
+        <v>null</v>
       </c>
       <c r="O49" t="str">
         <v>null</v>
@@ -4721,25 +4721,25 @@
         <v>null</v>
       </c>
       <c r="Q49" t="str">
-        <v>0</v>
+        <v>null</v>
       </c>
       <c r="R49" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S49" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/VolumeFlowRate</v>
       </c>
       <c r="T49" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0053</v>
       </c>
       <c r="U49" t="str">
         <v>null</v>
       </c>
       <c r="V49" t="str">
-        <v>minimum</v>
+        <v>null</v>
       </c>
       <c r="W49" t="str">
-        <v>true</v>
+        <v>null</v>
       </c>
       <c r="X49" t="str">
         <v>null</v>
@@ -4762,10 +4762,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_13</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
       </c>
       <c r="B50" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept|http://www.w3.org/ns/ssn/Property</v>
       </c>
       <c r="C50" t="str">
         <v>null</v>
@@ -4774,16 +4774,16 @@
         <v>null</v>
       </c>
       <c r="E50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="F50" t="str">
         <v>null</v>
       </c>
       <c r="G50" t="str">
-        <v>Biobedspuiwaterproductie S3 systeem</v>
+        <v>Zuurtegraad van het waswater</v>
       </c>
       <c r="H50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="I50" t="str">
         <v>null</v>
@@ -4798,10 +4798,10 @@
         <v>null</v>
       </c>
       <c r="M50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N50" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie</v>
+        <v>null</v>
       </c>
       <c r="O50" t="str">
         <v>null</v>
@@ -4810,25 +4810,25 @@
         <v>null</v>
       </c>
       <c r="Q50" t="str">
-        <v>0</v>
+        <v>null</v>
       </c>
       <c r="R50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
       <c r="S50" t="str">
-        <v>null</v>
+        <v>http://qudt.org/vocab/quantitykind/Acidity</v>
       </c>
       <c r="T50" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/fysico-chemisch/0076</v>
       </c>
       <c r="U50" t="str">
         <v>null</v>
       </c>
       <c r="V50" t="str">
-        <v>minimum</v>
+        <v>null</v>
       </c>
       <c r="W50" t="str">
-        <v>true</v>
+        <v>null</v>
       </c>
       <c r="X50" t="str">
         <v>null</v>
@@ -4851,7 +4851,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_14</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_1</v>
       </c>
       <c r="B51" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4869,7 +4869,7 @@
         <v>null</v>
       </c>
       <c r="G51" t="str">
-        <v>Biobedspoelwaterproductie S3 systeem</v>
+        <v>Zuurtegraad waswater S1 systeem</v>
       </c>
       <c r="H51" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -4887,19 +4887,19 @@
         <v>null</v>
       </c>
       <c r="M51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N51" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
       </c>
       <c r="O51" t="str">
-        <v>null</v>
+        <v>8.5</v>
       </c>
       <c r="P51" t="str">
         <v>null</v>
       </c>
       <c r="Q51" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R51" t="str">
         <v>null</v>
@@ -4914,7 +4914,7 @@
         <v>null</v>
       </c>
       <c r="V51" t="str">
-        <v>minimum</v>
+        <v>maximum</v>
       </c>
       <c r="W51" t="str">
         <v>true</v>
@@ -4940,7 +4940,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_15</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_10</v>
       </c>
       <c r="B52" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -4958,7 +4958,7 @@
         <v>null</v>
       </c>
       <c r="G52" t="str">
-        <v>Drukval S3 systeem</v>
+        <v>Drukval S2 systeem</v>
       </c>
       <c r="H52" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -4976,7 +4976,7 @@
         <v>null</v>
       </c>
       <c r="M52" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N52" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
@@ -5003,7 +5003,7 @@
         <v>null</v>
       </c>
       <c r="V52" t="str">
-        <v>maximum</v>
+        <v>exact</v>
       </c>
       <c r="W52" t="str">
         <v>true</v>
@@ -5029,7 +5029,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_16</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_11</v>
       </c>
       <c r="B53" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5047,7 +5047,7 @@
         <v>null</v>
       </c>
       <c r="G53" t="str">
-        <v>Geleidbaarheid waswater Lely Sphere systeem</v>
+        <v>Waswaterdebiet voorbevochtiging S3 systeem</v>
       </c>
       <c r="H53" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5065,10 +5065,10 @@
         <v>null</v>
       </c>
       <c r="M53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N53" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging</v>
       </c>
       <c r="O53" t="str">
         <v>null</v>
@@ -5092,7 +5092,7 @@
         <v>null</v>
       </c>
       <c r="V53" t="str">
-        <v>maximum</v>
+        <v>minimum</v>
       </c>
       <c r="W53" t="str">
         <v>true</v>
@@ -5118,7 +5118,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_17</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_12</v>
       </c>
       <c r="B54" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5136,7 +5136,7 @@
         <v>null</v>
       </c>
       <c r="G54" t="str">
-        <v>Waswaterdebiet Lely Sphere systeem</v>
+        <v>Waswaterdebiet bevloeiing S3 systeem</v>
       </c>
       <c r="H54" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5154,10 +5154,10 @@
         <v>null</v>
       </c>
       <c r="M54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N54" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing</v>
       </c>
       <c r="O54" t="str">
         <v>null</v>
@@ -5207,7 +5207,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_18</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_13</v>
       </c>
       <c r="B55" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5225,7 +5225,7 @@
         <v>null</v>
       </c>
       <c r="G55" t="str">
-        <v>Spuiwaterdebiet Lely Sphere systeem</v>
+        <v>Biobedspuiwaterproductie S3 systeem</v>
       </c>
       <c r="H55" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5243,10 +5243,10 @@
         <v>null</v>
       </c>
       <c r="M55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N55" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie</v>
       </c>
       <c r="O55" t="str">
         <v>null</v>
@@ -5296,7 +5296,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_19</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_14</v>
       </c>
       <c r="B56" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5314,7 +5314,7 @@
         <v>null</v>
       </c>
       <c r="G56" t="str">
-        <v>Elektriciteitsverbruik van de waswaterpomp(en) Lely Sphere systeem</v>
+        <v>Biobedspoelwaterproductie S3 systeem</v>
       </c>
       <c r="H56" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5332,10 +5332,10 @@
         <v>null</v>
       </c>
       <c r="M56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N56" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie</v>
       </c>
       <c r="O56" t="str">
         <v>null</v>
@@ -5385,7 +5385,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_15</v>
       </c>
       <c r="B57" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5403,7 +5403,7 @@
         <v>null</v>
       </c>
       <c r="G57" t="str">
-        <v>Geleidbaarheid waswater S1 systeem</v>
+        <v>Drukval S3 systeem</v>
       </c>
       <c r="H57" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5421,13 +5421,13 @@
         <v>null</v>
       </c>
       <c r="M57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="N57" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
       </c>
       <c r="O57" t="str">
-        <v>30</v>
+        <v>500</v>
       </c>
       <c r="P57" t="str">
         <v>null</v>
@@ -5474,7 +5474,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_16</v>
       </c>
       <c r="B58" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5492,7 +5492,7 @@
         <v>null</v>
       </c>
       <c r="G58" t="str">
-        <v>Waswaterdebiet S1 systeem</v>
+        <v>Geleidbaarheid waswater Lely Sphere systeem</v>
       </c>
       <c r="H58" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5510,10 +5510,10 @@
         <v>null</v>
       </c>
       <c r="M58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N58" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="O58" t="str">
         <v>null</v>
@@ -5537,7 +5537,7 @@
         <v>null</v>
       </c>
       <c r="V58" t="str">
-        <v>minimum</v>
+        <v>maximum</v>
       </c>
       <c r="W58" t="str">
         <v>true</v>
@@ -5563,7 +5563,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_4</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_17</v>
       </c>
       <c r="B59" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5581,7 +5581,7 @@
         <v>null</v>
       </c>
       <c r="G59" t="str">
-        <v>Spuiwaterdebiet S1 systeem</v>
+        <v>Waswaterdebiet Lely Sphere systeem</v>
       </c>
       <c r="H59" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5599,10 +5599,10 @@
         <v>null</v>
       </c>
       <c r="M59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N59" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
       </c>
       <c r="O59" t="str">
         <v>null</v>
@@ -5652,7 +5652,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_5</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_18</v>
       </c>
       <c r="B60" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5670,7 +5670,7 @@
         <v>null</v>
       </c>
       <c r="G60" t="str">
-        <v>Drukval S1 systeem</v>
+        <v>Spuiwaterdebiet Lely Sphere systeem</v>
       </c>
       <c r="H60" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5688,13 +5688,13 @@
         <v>null</v>
       </c>
       <c r="M60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N60" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
       </c>
       <c r="O60" t="str">
-        <v>500</v>
+        <v>null</v>
       </c>
       <c r="P60" t="str">
         <v>null</v>
@@ -5715,7 +5715,7 @@
         <v>null</v>
       </c>
       <c r="V60" t="str">
-        <v>exact</v>
+        <v>minimum</v>
       </c>
       <c r="W60" t="str">
         <v>true</v>
@@ -5741,7 +5741,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_6</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_19</v>
       </c>
       <c r="B61" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5759,7 +5759,7 @@
         <v>null</v>
       </c>
       <c r="G61" t="str">
-        <v>Zuurtegraad waswater S2 systeem</v>
+        <v>Elektriciteitsverbruik van de waswaterpomp(en) Lely Sphere systeem</v>
       </c>
       <c r="H61" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5777,13 +5777,13 @@
         <v>null</v>
       </c>
       <c r="M61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="N61" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
       </c>
       <c r="O61" t="str">
-        <v>14</v>
+        <v>null</v>
       </c>
       <c r="P61" t="str">
         <v>null</v>
@@ -5804,7 +5804,7 @@
         <v>null</v>
       </c>
       <c r="V61" t="str">
-        <v>maximum</v>
+        <v>minimum</v>
       </c>
       <c r="W61" t="str">
         <v>true</v>
@@ -5830,7 +5830,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_7</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_2</v>
       </c>
       <c r="B62" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5848,7 +5848,7 @@
         <v>null</v>
       </c>
       <c r="G62" t="str">
-        <v>Geleidbaarheid waswater S2 systeem</v>
+        <v>Geleidbaarheid waswater S1 systeem</v>
       </c>
       <c r="H62" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5866,13 +5866,13 @@
         <v>null</v>
       </c>
       <c r="M62" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N62" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="O62" t="str">
-        <v>500</v>
+        <v>30</v>
       </c>
       <c r="P62" t="str">
         <v>null</v>
@@ -5919,7 +5919,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_8</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_3</v>
       </c>
       <c r="B63" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -5937,7 +5937,7 @@
         <v>null</v>
       </c>
       <c r="G63" t="str">
-        <v>Waswaterdebiet S2 systeem</v>
+        <v>Waswaterdebiet S1 systeem</v>
       </c>
       <c r="H63" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -5955,7 +5955,7 @@
         <v>null</v>
       </c>
       <c r="M63" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N63" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
@@ -6008,7 +6008,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_9</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_4</v>
       </c>
       <c r="B64" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6026,7 +6026,7 @@
         <v>null</v>
       </c>
       <c r="G64" t="str">
-        <v>Spuiwaterdebiet S2 systeem</v>
+        <v>Spuiwaterdebiet S1 systeem</v>
       </c>
       <c r="H64" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
@@ -6044,7 +6044,7 @@
         <v>null</v>
       </c>
       <c r="M64" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N64" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
@@ -6097,7 +6097,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/in_gebruik</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_5</v>
       </c>
       <c r="B65" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6109,16 +6109,16 @@
         <v>null</v>
       </c>
       <c r="E65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="F65" t="str">
         <v>null</v>
       </c>
       <c r="G65" t="str">
-        <v>Stal in gebruik, dieren aanwezig.</v>
+        <v>Drukval S1 systeem</v>
       </c>
       <c r="H65" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="I65" t="str">
         <v>null</v>
@@ -6133,19 +6133,19 @@
         <v>null</v>
       </c>
       <c r="M65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="N65" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem</v>
       </c>
       <c r="O65" t="str">
-        <v>null</v>
+        <v>500</v>
       </c>
       <c r="P65" t="str">
         <v>null</v>
       </c>
       <c r="Q65" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R65" t="str">
         <v>null</v>
@@ -6160,10 +6160,10 @@
         <v>null</v>
       </c>
       <c r="V65" t="str">
-        <v>null</v>
+        <v>exact</v>
       </c>
       <c r="W65" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="X65" t="str">
         <v>null</v>
@@ -6186,7 +6186,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/leeg</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_6</v>
       </c>
       <c r="B66" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6198,16 +6198,16 @@
         <v>null</v>
       </c>
       <c r="E66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="F66" t="str">
         <v>null</v>
       </c>
       <c r="G66" t="str">
-        <v>Lege stal</v>
+        <v>Zuurtegraad waswater S2 systeem</v>
       </c>
       <c r="H66" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="I66" t="str">
         <v>null</v>
@@ -6222,19 +6222,19 @@
         <v>null</v>
       </c>
       <c r="M66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N66" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater</v>
       </c>
       <c r="O66" t="str">
-        <v>null</v>
+        <v>14</v>
       </c>
       <c r="P66" t="str">
         <v>null</v>
       </c>
       <c r="Q66" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R66" t="str">
         <v>null</v>
@@ -6249,10 +6249,10 @@
         <v>null</v>
       </c>
       <c r="V66" t="str">
-        <v>null</v>
+        <v>maximum</v>
       </c>
       <c r="W66" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="X66" t="str">
         <v>null</v>
@@ -6275,7 +6275,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/buiten_gebruik</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_7</v>
       </c>
       <c r="B67" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6287,16 +6287,16 @@
         <v>null</v>
       </c>
       <c r="E67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="F67" t="str">
         <v>null</v>
       </c>
       <c r="G67" t="str">
-        <v>Buiten gebruik</v>
+        <v>Geleidbaarheid waswater S2 systeem</v>
       </c>
       <c r="H67" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="I67" t="str">
         <v>null</v>
@@ -6311,19 +6311,19 @@
         <v>null</v>
       </c>
       <c r="M67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N67" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater</v>
       </c>
       <c r="O67" t="str">
-        <v>null</v>
+        <v>500</v>
       </c>
       <c r="P67" t="str">
         <v>null</v>
       </c>
       <c r="Q67" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R67" t="str">
         <v>null</v>
@@ -6338,10 +6338,10 @@
         <v>null</v>
       </c>
       <c r="V67" t="str">
-        <v>null</v>
+        <v>maximum</v>
       </c>
       <c r="W67" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="X67" t="str">
         <v>null</v>
@@ -6364,7 +6364,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/in_reiniging</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_8</v>
       </c>
       <c r="B68" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6376,16 +6376,16 @@
         <v>null</v>
       </c>
       <c r="E68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="F68" t="str">
         <v>null</v>
       </c>
       <c r="G68" t="str">
-        <v>In reiniging</v>
+        <v>Waswaterdebiet S2 systeem</v>
       </c>
       <c r="H68" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="I68" t="str">
         <v>null</v>
@@ -6400,10 +6400,10 @@
         <v>null</v>
       </c>
       <c r="M68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N68" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet</v>
       </c>
       <c r="O68" t="str">
         <v>null</v>
@@ -6412,7 +6412,7 @@
         <v>null</v>
       </c>
       <c r="Q68" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R68" t="str">
         <v>null</v>
@@ -6427,10 +6427,10 @@
         <v>null</v>
       </c>
       <c r="V68" t="str">
-        <v>null</v>
+        <v>minimum</v>
       </c>
       <c r="W68" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="X68" t="str">
         <v>null</v>
@@ -6453,7 +6453,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/onderhoud</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_9</v>
       </c>
       <c r="B69" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6465,16 +6465,16 @@
         <v>null</v>
       </c>
       <c r="E69" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="F69" t="str">
         <v>null</v>
       </c>
       <c r="G69" t="str">
-        <v>In onderhoud</v>
+        <v>Spuiwaterdebiet S2 systeem</v>
       </c>
       <c r="H69" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="I69" t="str">
         <v>null</v>
@@ -6489,10 +6489,10 @@
         <v>null</v>
       </c>
       <c r="M69" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="N69" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie</v>
       </c>
       <c r="O69" t="str">
         <v>null</v>
@@ -6501,7 +6501,7 @@
         <v>null</v>
       </c>
       <c r="Q69" t="str">
-        <v>null</v>
+        <v>0</v>
       </c>
       <c r="R69" t="str">
         <v>null</v>
@@ -6516,10 +6516,10 @@
         <v>null</v>
       </c>
       <c r="V69" t="str">
-        <v>null</v>
+        <v>minimum</v>
       </c>
       <c r="W69" t="str">
-        <v>null</v>
+        <v>true</v>
       </c>
       <c r="X69" t="str">
         <v>null</v>
@@ -6542,7 +6542,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/operationeel</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/in_gebruik</v>
       </c>
       <c r="B70" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6554,16 +6554,16 @@
         <v>null</v>
       </c>
       <c r="E70" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
       </c>
       <c r="F70" t="str">
         <v>null</v>
       </c>
       <c r="G70" t="str">
-        <v>Operationeel</v>
+        <v>Stal in gebruik, dieren aanwezig.</v>
       </c>
       <c r="H70" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
       </c>
       <c r="I70" t="str">
         <v>null</v>
@@ -6631,7 +6631,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/storing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/leeg</v>
       </c>
       <c r="B71" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6643,16 +6643,16 @@
         <v>null</v>
       </c>
       <c r="E71" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
       </c>
       <c r="F71" t="str">
         <v>null</v>
       </c>
       <c r="G71" t="str">
-        <v>Storing</v>
+        <v>Lege stal</v>
       </c>
       <c r="H71" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
       </c>
       <c r="I71" t="str">
         <v>null</v>
@@ -6720,7 +6720,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/enkelvoudig</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/buiten_gebruik</v>
       </c>
       <c r="B72" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6732,16 +6732,16 @@
         <v>null</v>
       </c>
       <c r="E72" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="F72" t="str">
         <v>null</v>
       </c>
       <c r="G72" t="str">
-        <v>Enkelvoudige opstelling</v>
+        <v>Buiten gebruik</v>
       </c>
       <c r="H72" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="I72" t="str">
         <v>null</v>
@@ -6809,7 +6809,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/gecombineerd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/in_reiniging</v>
       </c>
       <c r="B73" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6821,16 +6821,16 @@
         <v>null</v>
       </c>
       <c r="E73" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="F73" t="str">
         <v>null</v>
       </c>
       <c r="G73" t="str">
-        <v>Gecombineerde opstelling</v>
+        <v>In reiniging</v>
       </c>
       <c r="H73" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="I73" t="str">
         <v>null</v>
@@ -6898,7 +6898,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/onderhoud</v>
       </c>
       <c r="B74" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6910,16 +6910,16 @@
         <v>null</v>
       </c>
       <c r="E74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="F74" t="str">
-        <v>Lelysphere</v>
+        <v>null</v>
       </c>
       <c r="G74" t="str">
-        <v>Lely Sphere</v>
+        <v>In onderhoud</v>
       </c>
       <c r="H74" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="I74" t="str">
         <v>null</v>
@@ -6937,7 +6937,7 @@
         <v>null</v>
       </c>
       <c r="N74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
+        <v>null</v>
       </c>
       <c r="O74" t="str">
         <v>null</v>
@@ -6967,13 +6967,13 @@
         <v>null</v>
       </c>
       <c r="X74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="Y74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="Z74" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="AA74" t="str">
         <v>null</v>
@@ -6987,7 +6987,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/operationeel</v>
       </c>
       <c r="B75" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -6999,16 +6999,16 @@
         <v>null</v>
       </c>
       <c r="E75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="F75" t="str">
         <v>null</v>
       </c>
       <c r="G75" t="str">
-        <v>Luchtwassysteem</v>
+        <v>Operationeel</v>
       </c>
       <c r="H75" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="I75" t="str">
         <v>null</v>
@@ -7056,19 +7056,19 @@
         <v>null</v>
       </c>
       <c r="X75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="Y75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="Z75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="AA75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>null</v>
       </c>
       <c r="AB75" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
+        <v>null</v>
       </c>
       <c r="AC75" t="str">
         <v>null</v>
@@ -7076,7 +7076,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/storing</v>
       </c>
       <c r="B76" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7088,16 +7088,16 @@
         <v>null</v>
       </c>
       <c r="E76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="F76" t="str">
         <v>null</v>
       </c>
       <c r="G76" t="str">
-        <v>Luchtzuiveringssysteem</v>
+        <v>Storing</v>
       </c>
       <c r="H76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
       </c>
       <c r="I76" t="str">
         <v>null</v>
@@ -7151,13 +7151,13 @@
         <v>null</v>
       </c>
       <c r="Z76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="AA76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="AB76" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="AC76" t="str">
         <v>null</v>
@@ -7165,7 +7165,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/enkelvoudig</v>
       </c>
       <c r="B77" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7177,16 +7177,16 @@
         <v>null</v>
       </c>
       <c r="E77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
       </c>
       <c r="F77" t="str">
-        <v>S1</v>
+        <v>null</v>
       </c>
       <c r="G77" t="str">
-        <v>Biologisch luchtwassysteem</v>
+        <v>Enkelvoudige opstelling</v>
       </c>
       <c r="H77" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
       </c>
       <c r="I77" t="str">
         <v>null</v>
@@ -7204,7 +7204,7 @@
         <v>null</v>
       </c>
       <c r="N77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
+        <v>null</v>
       </c>
       <c r="O77" t="str">
         <v>null</v>
@@ -7234,13 +7234,13 @@
         <v>null</v>
       </c>
       <c r="X77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="Y77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="Z77" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="AA77" t="str">
         <v>null</v>
@@ -7254,7 +7254,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/gecombineerd</v>
       </c>
       <c r="B78" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7266,16 +7266,16 @@
         <v>null</v>
       </c>
       <c r="E78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
       </c>
       <c r="F78" t="str">
-        <v>S2</v>
+        <v>null</v>
       </c>
       <c r="G78" t="str">
-        <v>Chemisch luchtwassysteem</v>
+        <v>Gecombineerde opstelling</v>
       </c>
       <c r="H78" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
       </c>
       <c r="I78" t="str">
         <v>null</v>
@@ -7293,7 +7293,7 @@
         <v>null</v>
       </c>
       <c r="N78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
+        <v>null</v>
       </c>
       <c r="O78" t="str">
         <v>null</v>
@@ -7323,13 +7323,13 @@
         <v>null</v>
       </c>
       <c r="X78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
+        <v>null</v>
       </c>
       <c r="Y78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="Z78" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>null</v>
       </c>
       <c r="AA78" t="str">
         <v>null</v>
@@ -7343,7 +7343,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere</v>
       </c>
       <c r="B79" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7358,10 +7358,10 @@
         <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F79" t="str">
-        <v>S3</v>
+        <v>Lelysphere</v>
       </c>
       <c r="G79" t="str">
-        <v>Biobed</v>
+        <v>Lely Sphere</v>
       </c>
       <c r="H79" t="str">
         <v>null</v>
@@ -7382,7 +7382,7 @@
         <v>null</v>
       </c>
       <c r="N79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen</v>
       </c>
       <c r="O79" t="str">
         <v>null</v>
@@ -7412,13 +7412,13 @@
         <v>null</v>
       </c>
       <c r="X79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="Y79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Z79" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="AA79" t="str">
         <v>null</v>
@@ -7432,7 +7432,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k1</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="B80" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7441,28 +7441,28 @@
         <v>null</v>
       </c>
       <c r="D80" t="str">
-        <v>VLAREM klasse 1</v>
+        <v>null</v>
       </c>
       <c r="E80" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F80" t="str">
         <v>null</v>
       </c>
       <c r="G80" t="str">
-        <v>Klasse 1</v>
+        <v>Luchtwassysteem</v>
       </c>
       <c r="H80" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>null</v>
       </c>
       <c r="I80" t="str">
         <v>null</v>
       </c>
       <c r="J80" t="str">
-        <v>Indelingsklasse voor inrichtingen met de grootste milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 1 (zwaarste procedure).</v>
+        <v>null</v>
       </c>
       <c r="K80" t="str">
-        <v>Indelingsklasse voor inrichtingen met de grootste milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 1 (zwaarste procedure).</v>
+        <v>null</v>
       </c>
       <c r="L80" t="str">
         <v>null</v>
@@ -7501,19 +7501,19 @@
         <v>null</v>
       </c>
       <c r="X80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Y80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Z80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="AA80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="AB80" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="AC80" t="str">
         <v>null</v>
@@ -7521,7 +7521,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k2</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="B81" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7530,28 +7530,28 @@
         <v>null</v>
       </c>
       <c r="D81" t="str">
-        <v>VLAREM klasse 2</v>
+        <v>null</v>
       </c>
       <c r="E81" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F81" t="str">
         <v>null</v>
       </c>
       <c r="G81" t="str">
-        <v>Klasse 2</v>
+        <v>Luchtzuiveringssysteem</v>
       </c>
       <c r="H81" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="I81" t="str">
         <v>null</v>
       </c>
       <c r="J81" t="str">
-        <v>Indelingsklasse voor inrichtingen met een middelgrote milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 2.</v>
+        <v>null</v>
       </c>
       <c r="K81" t="str">
-        <v>Indelingsklasse voor inrichtingen met een middelgrote milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 2.</v>
+        <v>null</v>
       </c>
       <c r="L81" t="str">
         <v>null</v>
@@ -7596,13 +7596,13 @@
         <v>null</v>
       </c>
       <c r="Z81" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="AA81" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="AB81" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/lelysphere|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="AC81" t="str">
         <v>null</v>
@@ -7610,7 +7610,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k3</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s1</v>
       </c>
       <c r="B82" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
@@ -7619,28 +7619,28 @@
         <v>null</v>
       </c>
       <c r="D82" t="str">
-        <v>VLAREM klasse 3</v>
+        <v>null</v>
       </c>
       <c r="E82" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F82" t="str">
-        <v>null</v>
+        <v>S1</v>
       </c>
       <c r="G82" t="str">
-        <v>Klasse 3</v>
+        <v>Biologisch luchtwassysteem</v>
       </c>
       <c r="H82" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>null</v>
       </c>
       <c r="I82" t="str">
         <v>null</v>
       </c>
       <c r="J82" t="str">
-        <v>Indelingsklasse voor inrichtingen met een beperkte milieu-impact. Voor deze activiteiten geldt een meldingsplicht (klasse 3).</v>
+        <v>null</v>
       </c>
       <c r="K82" t="str">
-        <v>Indelingsklasse voor inrichtingen met een beperkte milieu-impact. Voor deze activiteiten geldt een meldingsplicht (klasse 3).</v>
+        <v>null</v>
       </c>
       <c r="L82" t="str">
         <v>null</v>
@@ -7649,7 +7649,7 @@
         <v>null</v>
       </c>
       <c r="N82" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
       <c r="O82" t="str">
         <v>null</v>
@@ -7679,13 +7679,13 @@
         <v>null</v>
       </c>
       <c r="X82" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="Y82" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Z82" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="AA82" t="str">
         <v>null</v>
@@ -7699,10 +7699,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/dataleverancierstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s2</v>
       </c>
       <c r="B83" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C83" t="str">
         <v>null</v>
@@ -7711,13 +7711,13 @@
         <v>null</v>
       </c>
       <c r="E83" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F83" t="str">
-        <v>null</v>
+        <v>S2</v>
       </c>
       <c r="G83" t="str">
-        <v>conceptschema dataleverancier status</v>
+        <v>Chemisch luchtwassysteem</v>
       </c>
       <c r="H83" t="str">
         <v>null</v>
@@ -7738,7 +7738,7 @@
         <v>null</v>
       </c>
       <c r="N83" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
       <c r="O83" t="str">
         <v>null</v>
@@ -7768,13 +7768,13 @@
         <v>null</v>
       </c>
       <c r="X83" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem</v>
       </c>
       <c r="Y83" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Z83" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtwassysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="AA83" t="str">
         <v>null</v>
@@ -7783,15 +7783,15 @@
         <v>null</v>
       </c>
       <c r="AC83" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/gevalideerd|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/geweigerd|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/ingetrokken|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/nietgevalideerd</v>
+        <v>null</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/medium</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/s3</v>
       </c>
       <c r="B84" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C84" t="str">
         <v>null</v>
@@ -7800,13 +7800,13 @@
         <v>null</v>
       </c>
       <c r="E84" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
       </c>
       <c r="F84" t="str">
-        <v>null</v>
+        <v>S3</v>
       </c>
       <c r="G84" t="str">
-        <v>conceptschema luchtzuiveringssysteem medium</v>
+        <v>Biobed</v>
       </c>
       <c r="H84" t="str">
         <v>null</v>
@@ -7827,7 +7827,7 @@
         <v>null</v>
       </c>
       <c r="N84" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
       <c r="O84" t="str">
         <v>null</v>
@@ -7857,13 +7857,13 @@
         <v>null</v>
       </c>
       <c r="X84" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Y84" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="Z84" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
       </c>
       <c r="AA84" t="str">
         <v>null</v>
@@ -7872,42 +7872,42 @@
         <v>null</v>
       </c>
       <c r="AC84" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/hetelektronischmonitoringssysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/lucht|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/stal|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
+        <v>null</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k1</v>
       </c>
       <c r="B85" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C85" t="str">
         <v>null</v>
       </c>
       <c r="D85" t="str">
-        <v>Ranges</v>
+        <v>VLAREM klasse 1</v>
       </c>
       <c r="E85" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="F85" t="str">
         <v>null</v>
       </c>
       <c r="G85" t="str">
-        <v>conceptschema luchtzuiveringssysteem normbandbreedte</v>
+        <v>Klasse 1</v>
       </c>
       <c r="H85" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="I85" t="str">
         <v>null</v>
       </c>
       <c r="J85" t="str">
-        <v>null</v>
+        <v>Indelingsklasse voor inrichtingen met de grootste milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 1 (zwaarste procedure).</v>
       </c>
       <c r="K85" t="str">
-        <v>null</v>
+        <v>Indelingsklasse voor inrichtingen met de grootste milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 1 (zwaarste procedure).</v>
       </c>
       <c r="L85" t="str">
         <v>null</v>
@@ -7961,42 +7961,42 @@
         <v>null</v>
       </c>
       <c r="AC85" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_10|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_11|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_12|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_13|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_14|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_15|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_16|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_1|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_2|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_3|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_4|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_5|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_6|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_7|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_8|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_9</v>
+        <v>null</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k2</v>
       </c>
       <c r="B86" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C86" t="str">
         <v>null</v>
       </c>
       <c r="D86" t="str">
-        <v>null</v>
+        <v>VLAREM klasse 2</v>
       </c>
       <c r="E86" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="F86" t="str">
         <v>null</v>
       </c>
       <c r="G86" t="str">
-        <v>conceptschema luchtzuiveringssysteem eigenschap</v>
+        <v>Klasse 2</v>
       </c>
       <c r="H86" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="I86" t="str">
         <v>null</v>
       </c>
       <c r="J86" t="str">
-        <v>null</v>
+        <v>Indelingsklasse voor inrichtingen met een middelgrote milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 2.</v>
       </c>
       <c r="K86" t="str">
-        <v>null</v>
+        <v>Indelingsklasse voor inrichtingen met een middelgrote milieu-impact. Voor deze activiteiten geldt een omgevingsvergunning klasse 2.</v>
       </c>
       <c r="L86" t="str">
         <v>null</v>
@@ -8050,42 +8050,42 @@
         <v>null</v>
       </c>
       <c r="AC86" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
+        <v>null</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k3</v>
       </c>
       <c r="B87" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C87" t="str">
         <v>null</v>
       </c>
       <c r="D87" t="str">
-        <v>null</v>
+        <v>VLAREM klasse 3</v>
       </c>
       <c r="E87" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="F87" t="str">
         <v>null</v>
       </c>
       <c r="G87" t="str">
-        <v>conceptschema luchtzuiveringssysteem parameter specificatie</v>
+        <v>Klasse 3</v>
       </c>
       <c r="H87" t="str">
-        <v>null</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
       </c>
       <c r="I87" t="str">
         <v>null</v>
       </c>
       <c r="J87" t="str">
-        <v>Het schema van indelingsklassen (1, 2, 3) zoals vastgelegd in de Vlaamse milieuregelgeving (VLAREM).</v>
+        <v>Indelingsklasse voor inrichtingen met een beperkte milieu-impact. Voor deze activiteiten geldt een meldingsplicht (klasse 3).</v>
       </c>
       <c r="K87" t="str">
-        <v>Het schema van indelingsklassen (1, 2, 3) zoals vastgelegd in de Vlaamse milieuregelgeving (VLAREM).</v>
+        <v>Indelingsklasse voor inrichtingen met een beperkte milieu-impact. Voor deze activiteiten geldt een meldingsplicht (klasse 3).</v>
       </c>
       <c r="L87" t="str">
         <v>null</v>
@@ -8139,12 +8139,12 @@
         <v>null</v>
       </c>
       <c r="AC87" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_10|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_11|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_12|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_13|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_14|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_15|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_16|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_17|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_18|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_19|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_1|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_2|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_3|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_4|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_5|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_6|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_7|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_8|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_9</v>
+        <v>null</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/dataleverancierstatus</v>
       </c>
       <c r="B88" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -8162,7 +8162,7 @@
         <v>null</v>
       </c>
       <c r="G88" t="str">
-        <v>conceptschema luchtzuiveringssysteem stalbezetting</v>
+        <v>conceptschema dataleverancier status</v>
       </c>
       <c r="H88" t="str">
         <v>null</v>
@@ -8228,12 +8228,12 @@
         <v>null</v>
       </c>
       <c r="AC88" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/in_gebruik|https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/leeg</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/gevalideerd|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/geweigerd|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/ingetrokken|https://data.omgeving.vlaanderen.be/id/concept/lzs/dataleverancierstatus/nietgevalideerd</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/medium</v>
       </c>
       <c r="B89" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -8251,7 +8251,7 @@
         <v>null</v>
       </c>
       <c r="G89" t="str">
-        <v>conceptschema  luchtzuiveringssysteem opstelingen</v>
+        <v>conceptschema luchtzuiveringssysteem medium</v>
       </c>
       <c r="H89" t="str">
         <v>null</v>
@@ -8317,12 +8317,12 @@
         <v>null</v>
       </c>
       <c r="AC89" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/enkelvoudig|https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/gecombineerd</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/hetelektronischmonitoringssysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/lucht|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/spuiwater|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/stal|https://data.omgeving.vlaanderen.be/id/concept/lzs/medium/waswater</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/norm-bandbreedte</v>
       </c>
       <c r="B90" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -8331,7 +8331,7 @@
         <v>null</v>
       </c>
       <c r="D90" t="str">
-        <v>null</v>
+        <v>Ranges</v>
       </c>
       <c r="E90" t="str">
         <v>null</v>
@@ -8340,7 +8340,7 @@
         <v>null</v>
       </c>
       <c r="G90" t="str">
-        <v>conceptschema luchtzuiveringssysteem status</v>
+        <v>conceptschema luchtzuiveringssysteem normbandbreedte</v>
       </c>
       <c r="H90" t="str">
         <v>null</v>
@@ -8406,12 +8406,12 @@
         <v>null</v>
       </c>
       <c r="AC90" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/buiten_gebruik|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/in_reiniging|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/onderhoud|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/operationeel|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/storing</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_10|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_11|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_12|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_13|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_14|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_15|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_16|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_17|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_18|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_19|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_1|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_20|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_21|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_2|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_3|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_4|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_5|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_6|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_7|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_8|https://data.omgeving.vlaanderen.be/id/concept/lzs/norm_bandbreedte/_9</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter</v>
       </c>
       <c r="B91" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -8429,7 +8429,7 @@
         <v>null</v>
       </c>
       <c r="G91" t="str">
-        <v>conceptschema luchtzuiveringssysteem</v>
+        <v>conceptschema luchtzuiveringssysteem eigenschap</v>
       </c>
       <c r="H91" t="str">
         <v>null</v>
@@ -8495,12 +8495,12 @@
         <v>null</v>
       </c>
       <c r="AC91" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebiet|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/spuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/drukvaloverhetsysteem|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietvoorbevochtiging|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/waswaterdebietbevloeiing|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/geleidbaarheidvanhetwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/zuurtegraadwaswater|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/elektriciteitsverbruikwaterpompen|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspoelwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/biobedspuiwaterproductie|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/stalbezetting|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter/systeemstatus</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/parameter-norm</v>
       </c>
       <c r="B92" t="str">
         <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
@@ -8518,78 +8518,523 @@
         <v>null</v>
       </c>
       <c r="G92" t="str">
+        <v>conceptschema luchtzuiveringssysteem parameter specificatie</v>
+      </c>
+      <c r="H92" t="str">
+        <v>null</v>
+      </c>
+      <c r="I92" t="str">
+        <v>null</v>
+      </c>
+      <c r="J92" t="str">
+        <v>Het schema van indelingsklassen (1, 2, 3) zoals vastgelegd in de Vlaamse milieuregelgeving (VLAREM).</v>
+      </c>
+      <c r="K92" t="str">
+        <v>Het schema van indelingsklassen (1, 2, 3) zoals vastgelegd in de Vlaamse milieuregelgeving (VLAREM).</v>
+      </c>
+      <c r="L92" t="str">
+        <v>null</v>
+      </c>
+      <c r="M92" t="str">
+        <v>null</v>
+      </c>
+      <c r="N92" t="str">
+        <v>null</v>
+      </c>
+      <c r="O92" t="str">
+        <v>null</v>
+      </c>
+      <c r="P92" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q92" t="str">
+        <v>null</v>
+      </c>
+      <c r="R92" t="str">
+        <v>null</v>
+      </c>
+      <c r="S92" t="str">
+        <v>null</v>
+      </c>
+      <c r="T92" t="str">
+        <v>null</v>
+      </c>
+      <c r="U92" t="str">
+        <v>null</v>
+      </c>
+      <c r="V92" t="str">
+        <v>null</v>
+      </c>
+      <c r="W92" t="str">
+        <v>null</v>
+      </c>
+      <c r="X92" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y92" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z92" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA92" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB92" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC92" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_10|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_11|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_12|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_13|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_14|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_15|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_16|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_17|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_18|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_19|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_1|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_2|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_3|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_4|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_5|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_6|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_7|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_8|https://data.omgeving.vlaanderen.be/id/concept/lzs/parameter_norm/_9</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/stalbezetting</v>
+      </c>
+      <c r="B93" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C93" t="str">
+        <v>null</v>
+      </c>
+      <c r="D93" t="str">
+        <v>null</v>
+      </c>
+      <c r="E93" t="str">
+        <v>null</v>
+      </c>
+      <c r="F93" t="str">
+        <v>null</v>
+      </c>
+      <c r="G93" t="str">
+        <v>conceptschema luchtzuiveringssysteem stalbezetting</v>
+      </c>
+      <c r="H93" t="str">
+        <v>null</v>
+      </c>
+      <c r="I93" t="str">
+        <v>null</v>
+      </c>
+      <c r="J93" t="str">
+        <v>null</v>
+      </c>
+      <c r="K93" t="str">
+        <v>null</v>
+      </c>
+      <c r="L93" t="str">
+        <v>null</v>
+      </c>
+      <c r="M93" t="str">
+        <v>null</v>
+      </c>
+      <c r="N93" t="str">
+        <v>null</v>
+      </c>
+      <c r="O93" t="str">
+        <v>null</v>
+      </c>
+      <c r="P93" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q93" t="str">
+        <v>null</v>
+      </c>
+      <c r="R93" t="str">
+        <v>null</v>
+      </c>
+      <c r="S93" t="str">
+        <v>null</v>
+      </c>
+      <c r="T93" t="str">
+        <v>null</v>
+      </c>
+      <c r="U93" t="str">
+        <v>null</v>
+      </c>
+      <c r="V93" t="str">
+        <v>null</v>
+      </c>
+      <c r="W93" t="str">
+        <v>null</v>
+      </c>
+      <c r="X93" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y93" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z93" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA93" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB93" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC93" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/in_gebruik|https://data.omgeving.vlaanderen.be/id/concept/lzs/stalbezetting/leeg</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemopstelling</v>
+      </c>
+      <c r="B94" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C94" t="str">
+        <v>null</v>
+      </c>
+      <c r="D94" t="str">
+        <v>null</v>
+      </c>
+      <c r="E94" t="str">
+        <v>null</v>
+      </c>
+      <c r="F94" t="str">
+        <v>null</v>
+      </c>
+      <c r="G94" t="str">
+        <v>conceptschema  luchtzuiveringssysteem opstelingen</v>
+      </c>
+      <c r="H94" t="str">
+        <v>null</v>
+      </c>
+      <c r="I94" t="str">
+        <v>null</v>
+      </c>
+      <c r="J94" t="str">
+        <v>null</v>
+      </c>
+      <c r="K94" t="str">
+        <v>null</v>
+      </c>
+      <c r="L94" t="str">
+        <v>null</v>
+      </c>
+      <c r="M94" t="str">
+        <v>null</v>
+      </c>
+      <c r="N94" t="str">
+        <v>null</v>
+      </c>
+      <c r="O94" t="str">
+        <v>null</v>
+      </c>
+      <c r="P94" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q94" t="str">
+        <v>null</v>
+      </c>
+      <c r="R94" t="str">
+        <v>null</v>
+      </c>
+      <c r="S94" t="str">
+        <v>null</v>
+      </c>
+      <c r="T94" t="str">
+        <v>null</v>
+      </c>
+      <c r="U94" t="str">
+        <v>null</v>
+      </c>
+      <c r="V94" t="str">
+        <v>null</v>
+      </c>
+      <c r="W94" t="str">
+        <v>null</v>
+      </c>
+      <c r="X94" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y94" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z94" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA94" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB94" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC94" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/enkelvoudig|https://data.omgeving.vlaanderen.be/id/concept/lzs/systeemopstelling/gecombineerd</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemstatus</v>
+      </c>
+      <c r="B95" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C95" t="str">
+        <v>null</v>
+      </c>
+      <c r="D95" t="str">
+        <v>null</v>
+      </c>
+      <c r="E95" t="str">
+        <v>null</v>
+      </c>
+      <c r="F95" t="str">
+        <v>null</v>
+      </c>
+      <c r="G95" t="str">
+        <v>conceptschema luchtzuiveringssysteem status</v>
+      </c>
+      <c r="H95" t="str">
+        <v>null</v>
+      </c>
+      <c r="I95" t="str">
+        <v>null</v>
+      </c>
+      <c r="J95" t="str">
+        <v>null</v>
+      </c>
+      <c r="K95" t="str">
+        <v>null</v>
+      </c>
+      <c r="L95" t="str">
+        <v>null</v>
+      </c>
+      <c r="M95" t="str">
+        <v>null</v>
+      </c>
+      <c r="N95" t="str">
+        <v>null</v>
+      </c>
+      <c r="O95" t="str">
+        <v>null</v>
+      </c>
+      <c r="P95" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q95" t="str">
+        <v>null</v>
+      </c>
+      <c r="R95" t="str">
+        <v>null</v>
+      </c>
+      <c r="S95" t="str">
+        <v>null</v>
+      </c>
+      <c r="T95" t="str">
+        <v>null</v>
+      </c>
+      <c r="U95" t="str">
+        <v>null</v>
+      </c>
+      <c r="V95" t="str">
+        <v>null</v>
+      </c>
+      <c r="W95" t="str">
+        <v>null</v>
+      </c>
+      <c r="X95" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y95" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z95" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA95" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB95" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC95" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/status/buiten_gebruik|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/in_reiniging|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/onderhoud|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/operationeel|https://data.omgeving.vlaanderen.be/id/concept/lzs/status/storing</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/lzs/systeemtype</v>
+      </c>
+      <c r="B96" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C96" t="str">
+        <v>null</v>
+      </c>
+      <c r="D96" t="str">
+        <v>null</v>
+      </c>
+      <c r="E96" t="str">
+        <v>null</v>
+      </c>
+      <c r="F96" t="str">
+        <v>null</v>
+      </c>
+      <c r="G96" t="str">
+        <v>conceptschema luchtzuiveringssysteem</v>
+      </c>
+      <c r="H96" t="str">
+        <v>null</v>
+      </c>
+      <c r="I96" t="str">
+        <v>null</v>
+      </c>
+      <c r="J96" t="str">
+        <v>null</v>
+      </c>
+      <c r="K96" t="str">
+        <v>null</v>
+      </c>
+      <c r="L96" t="str">
+        <v>null</v>
+      </c>
+      <c r="M96" t="str">
+        <v>null</v>
+      </c>
+      <c r="N96" t="str">
+        <v>null</v>
+      </c>
+      <c r="O96" t="str">
+        <v>null</v>
+      </c>
+      <c r="P96" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q96" t="str">
+        <v>null</v>
+      </c>
+      <c r="R96" t="str">
+        <v>null</v>
+      </c>
+      <c r="S96" t="str">
+        <v>null</v>
+      </c>
+      <c r="T96" t="str">
+        <v>null</v>
+      </c>
+      <c r="U96" t="str">
+        <v>null</v>
+      </c>
+      <c r="V96" t="str">
+        <v>null</v>
+      </c>
+      <c r="W96" t="str">
+        <v>null</v>
+      </c>
+      <c r="X96" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y96" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z96" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA96" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB96" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC96" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/concept/lzs/type/luchtzuiveringssysteem</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>https://data.omgeving.vlaanderen.be/id/conceptscheme/vlarem-klasse</v>
+      </c>
+      <c r="B97" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
+      </c>
+      <c r="C97" t="str">
+        <v>null</v>
+      </c>
+      <c r="D97" t="str">
+        <v>null</v>
+      </c>
+      <c r="E97" t="str">
+        <v>null</v>
+      </c>
+      <c r="F97" t="str">
+        <v>null</v>
+      </c>
+      <c r="G97" t="str">
         <v>VLAREM indelingsklassen</v>
       </c>
-      <c r="H92" t="str">
-        <v>null</v>
-      </c>
-      <c r="I92" t="str">
-        <v>null</v>
-      </c>
-      <c r="J92" t="str">
-        <v>null</v>
-      </c>
-      <c r="K92" t="str">
-        <v>null</v>
-      </c>
-      <c r="L92" t="str">
-        <v>null</v>
-      </c>
-      <c r="M92" t="str">
-        <v>null</v>
-      </c>
-      <c r="N92" t="str">
-        <v>null</v>
-      </c>
-      <c r="O92" t="str">
-        <v>null</v>
-      </c>
-      <c r="P92" t="str">
-        <v>null</v>
-      </c>
-      <c r="Q92" t="str">
-        <v>null</v>
-      </c>
-      <c r="R92" t="str">
-        <v>null</v>
-      </c>
-      <c r="S92" t="str">
-        <v>null</v>
-      </c>
-      <c r="T92" t="str">
-        <v>null</v>
-      </c>
-      <c r="U92" t="str">
-        <v>null</v>
-      </c>
-      <c r="V92" t="str">
-        <v>null</v>
-      </c>
-      <c r="W92" t="str">
-        <v>null</v>
-      </c>
-      <c r="X92" t="str">
-        <v>null</v>
-      </c>
-      <c r="Y92" t="str">
-        <v>null</v>
-      </c>
-      <c r="Z92" t="str">
-        <v>null</v>
-      </c>
-      <c r="AA92" t="str">
-        <v>null</v>
-      </c>
-      <c r="AB92" t="str">
-        <v>null</v>
-      </c>
-      <c r="AC92" t="str">
+      <c r="H97" t="str">
+        <v>null</v>
+      </c>
+      <c r="I97" t="str">
+        <v>null</v>
+      </c>
+      <c r="J97" t="str">
+        <v>null</v>
+      </c>
+      <c r="K97" t="str">
+        <v>null</v>
+      </c>
+      <c r="L97" t="str">
+        <v>null</v>
+      </c>
+      <c r="M97" t="str">
+        <v>null</v>
+      </c>
+      <c r="N97" t="str">
+        <v>null</v>
+      </c>
+      <c r="O97" t="str">
+        <v>null</v>
+      </c>
+      <c r="P97" t="str">
+        <v>null</v>
+      </c>
+      <c r="Q97" t="str">
+        <v>null</v>
+      </c>
+      <c r="R97" t="str">
+        <v>null</v>
+      </c>
+      <c r="S97" t="str">
+        <v>null</v>
+      </c>
+      <c r="T97" t="str">
+        <v>null</v>
+      </c>
+      <c r="U97" t="str">
+        <v>null</v>
+      </c>
+      <c r="V97" t="str">
+        <v>null</v>
+      </c>
+      <c r="W97" t="str">
+        <v>null</v>
+      </c>
+      <c r="X97" t="str">
+        <v>null</v>
+      </c>
+      <c r="Y97" t="str">
+        <v>null</v>
+      </c>
+      <c r="Z97" t="str">
+        <v>null</v>
+      </c>
+      <c r="AA97" t="str">
+        <v>null</v>
+      </c>
+      <c r="AB97" t="str">
+        <v>null</v>
+      </c>
+      <c r="AC97" t="str">
         <v>https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k1|https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k2|https://data.omgeving.vlaanderen.be/id/concept/vlarem-klasse/k3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC97"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>